<commit_message>
Update VO manifest generation to include latest dialogues and replace celebration line with unregistered prompt
</commit_message>
<xml_diff>
--- a/HI02H04_L02_S01_dist/VO_Manifest.xlsx
+++ b/HI02H04_L02_S01_dist/VO_Manifest.xlsx
@@ -1185,12 +1185,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>vo_celebrate</t>
+          <t>vo_cel_prompt</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>शाबाश! आपने पूरी कहानी ध्यान से पढ़ी और सभी प्रश्नों के उत्तर दे दिए।</t>
+          <t>बहुत बढ़िया, दोस्त! तुमने कमाल कर दिया!</t>
         </is>
       </c>
     </row>

</xml_diff>